<commit_message>
Day 2 curriculum tracking
</commit_message>
<xml_diff>
--- a/12603676.xlsx
+++ b/12603676.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MCA\py\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6DB6367-8D31-4B69-BDA2-F7E3743EE33E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5984879C-5B25-45AC-9B13-898CD66A6439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1018,25 +1018,47 @@
       <c r="N6" s="12"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="15" t="str">
+      <c r="A7" s="8">
+        <v>46246</v>
+      </c>
+      <c r="B7" s="14">
+        <v>140</v>
+      </c>
+      <c r="C7" s="14">
+        <v>10</v>
+      </c>
+      <c r="D7" s="14">
+        <v>40</v>
+      </c>
+      <c r="E7" s="14">
+        <v>0</v>
+      </c>
+      <c r="F7" s="14">
+        <v>350</v>
+      </c>
+      <c r="G7" s="14">
+        <v>7</v>
+      </c>
+      <c r="H7" s="14">
+        <v>120</v>
+      </c>
+      <c r="I7" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
+        <v>780</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N7" s="17"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
long time no see
</commit_message>
<xml_diff>
--- a/12603676.xlsx
+++ b/12603676.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MCA\py\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5984879C-5B25-45AC-9B13-898CD66A6439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A86E466F-71D1-43AE-B549-931020BAC96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -197,6 +197,21 @@
   </si>
   <si>
     <t>CAP776</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Satisfied</t>
+  </si>
+  <si>
+    <t>High</t>
   </si>
 </sst>
 </file>
@@ -1062,861 +1077,1719 @@
       <c r="N7" s="17"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+      <c r="A8" s="8">
+        <v>46247</v>
+      </c>
+      <c r="B8" s="14">
+        <v>300</v>
+      </c>
+      <c r="C8" s="14">
+        <v>10</v>
+      </c>
+      <c r="D8" s="14">
+        <v>40</v>
+      </c>
+      <c r="E8" s="14">
+        <v>30</v>
+      </c>
+      <c r="F8" s="14">
+        <v>300</v>
+      </c>
+      <c r="G8" s="14">
+        <v>6</v>
+      </c>
+      <c r="H8" s="14">
+        <v>100</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>780</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
+        <v>660</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N8" s="17"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="A9" s="8">
+        <v>46248</v>
+      </c>
+      <c r="B9" s="14">
+        <v>360</v>
+      </c>
+      <c r="C9" s="14">
+        <v>10</v>
+      </c>
+      <c r="D9" s="14">
+        <v>30</v>
+      </c>
+      <c r="E9" s="14">
+        <v>30</v>
+      </c>
+      <c r="F9" s="14">
+        <v>200</v>
+      </c>
+      <c r="G9" s="14">
+        <v>4</v>
+      </c>
+      <c r="H9" s="14">
+        <v>250</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>880</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
+        <v>560</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N9" s="17"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+      <c r="A10" s="8">
+        <v>46249</v>
+      </c>
+      <c r="B10" s="14">
+        <v>420</v>
+      </c>
+      <c r="C10" s="14">
+        <v>10</v>
+      </c>
+      <c r="D10" s="14">
+        <v>40</v>
+      </c>
+      <c r="E10" s="14">
+        <v>30</v>
+      </c>
+      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>120</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>620</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
+        <v>820</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N10" s="17"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="15" t="str">
+      <c r="A11" s="8">
+        <v>46250</v>
+      </c>
+      <c r="B11" s="14">
+        <v>360</v>
+      </c>
+      <c r="C11" s="14">
+        <v>0</v>
+      </c>
+      <c r="D11" s="14">
+        <v>40</v>
+      </c>
+      <c r="E11" s="14">
+        <v>30</v>
+      </c>
+      <c r="F11" s="14">
+        <v>0</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14">
+        <v>200</v>
+      </c>
+      <c r="I11" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="15" t="str">
+        <v>630</v>
+      </c>
+      <c r="J11" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
+        <v>810</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N11" s="17"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+      <c r="A12" s="8">
+        <v>46251</v>
+      </c>
+      <c r="B12" s="14">
+        <v>360</v>
+      </c>
+      <c r="C12" s="14">
+        <v>10</v>
+      </c>
+      <c r="D12" s="14">
+        <v>40</v>
+      </c>
+      <c r="E12" s="14">
+        <v>30</v>
+      </c>
+      <c r="F12" s="14">
+        <v>250</v>
+      </c>
+      <c r="G12" s="14">
+        <v>5</v>
+      </c>
+      <c r="H12" s="14">
+        <v>250</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>940</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
+        <v>500</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N12" s="17"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="A13" s="8">
+        <v>46252</v>
+      </c>
+      <c r="B13" s="14">
+        <v>300</v>
+      </c>
+      <c r="C13" s="14">
+        <v>90</v>
+      </c>
+      <c r="D13" s="14">
+        <v>50</v>
+      </c>
+      <c r="E13" s="14">
+        <v>30</v>
+      </c>
+      <c r="F13" s="14">
+        <v>350</v>
+      </c>
+      <c r="G13" s="14">
+        <v>7</v>
+      </c>
+      <c r="H13" s="14">
+        <v>300</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1120</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
+        <v>320</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N13" s="17"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="8">
+        <v>46253</v>
+      </c>
+      <c r="B14" s="14">
+        <v>360</v>
+      </c>
+      <c r="C14" s="14">
+        <v>100</v>
+      </c>
+      <c r="D14" s="14">
+        <v>40</v>
+      </c>
+      <c r="E14" s="14">
+        <v>30</v>
+      </c>
+      <c r="F14" s="14">
+        <v>300</v>
+      </c>
+      <c r="G14" s="14">
+        <v>6</v>
+      </c>
+      <c r="H14" s="14">
+        <v>120</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="8">
+        <v>46254</v>
+      </c>
+      <c r="B15" s="14">
+        <v>140</v>
+      </c>
+      <c r="C15" s="14">
+        <v>90</v>
+      </c>
+      <c r="D15" s="14">
+        <v>40</v>
+      </c>
+      <c r="E15" s="14">
+        <v>30</v>
+      </c>
+      <c r="F15" s="14">
+        <v>200</v>
+      </c>
+      <c r="G15" s="14">
+        <v>4</v>
+      </c>
+      <c r="H15" s="14">
+        <v>100</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+        <v>840</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="A16" s="8">
+        <v>46255</v>
+      </c>
+      <c r="B16" s="14">
+        <v>420</v>
+      </c>
+      <c r="C16" s="14">
+        <v>120</v>
+      </c>
+      <c r="D16" s="14">
+        <v>100</v>
+      </c>
+      <c r="E16" s="14">
+        <v>30</v>
+      </c>
+      <c r="F16" s="14">
+        <v>250</v>
+      </c>
+      <c r="G16" s="14">
+        <v>5</v>
+      </c>
+      <c r="H16" s="14">
+        <v>120</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="A17" s="8">
+        <v>46256</v>
+      </c>
+      <c r="B17" s="14">
+        <v>420</v>
+      </c>
+      <c r="C17" s="14">
+        <v>70</v>
+      </c>
+      <c r="D17" s="14">
+        <v>40</v>
+      </c>
+      <c r="E17" s="14">
+        <v>0</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14">
+        <v>120</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>650</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
+        <v>790</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="8">
+        <v>46257</v>
+      </c>
+      <c r="B18" s="14">
+        <v>360</v>
+      </c>
+      <c r="C18" s="14">
+        <v>0</v>
+      </c>
+      <c r="D18" s="14">
+        <v>40</v>
+      </c>
+      <c r="E18" s="14">
+        <v>30</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14">
+        <v>90</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>520</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
+        <v>920</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="8">
+        <v>46258</v>
+      </c>
+      <c r="B19" s="14">
+        <v>300</v>
+      </c>
+      <c r="C19" s="14">
+        <v>120</v>
+      </c>
+      <c r="D19" s="14">
+        <v>0</v>
+      </c>
+      <c r="E19" s="14">
+        <v>0</v>
+      </c>
+      <c r="F19" s="14">
+        <v>250</v>
+      </c>
+      <c r="G19" s="14">
+        <v>5</v>
+      </c>
+      <c r="H19" s="14">
+        <v>10</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>680</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
+        <v>760</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N19" s="17"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="8">
+        <v>46259</v>
+      </c>
+      <c r="B20" s="14">
+        <v>300</v>
+      </c>
+      <c r="C20" s="14">
+        <v>120</v>
+      </c>
+      <c r="D20" s="14">
+        <v>60</v>
+      </c>
+      <c r="E20" s="14">
+        <v>50</v>
+      </c>
+      <c r="F20" s="14">
+        <v>250</v>
+      </c>
+      <c r="G20" s="14">
+        <v>5</v>
+      </c>
+      <c r="H20" s="14">
+        <v>120</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
+        <v>540</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>55</v>
+      </c>
       <c r="N20" s="17"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="8">
+        <v>46260</v>
+      </c>
+      <c r="B21" s="14">
+        <v>300</v>
+      </c>
+      <c r="C21" s="14">
+        <v>110</v>
+      </c>
+      <c r="D21" s="14">
+        <v>60</v>
+      </c>
+      <c r="E21" s="14">
+        <v>50</v>
+      </c>
+      <c r="F21" s="14">
+        <v>300</v>
+      </c>
+      <c r="G21" s="14">
+        <v>6</v>
+      </c>
+      <c r="H21" s="14">
+        <v>120</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>940</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
+        <v>500</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="8">
+        <v>46261</v>
+      </c>
+      <c r="B22" s="14">
+        <v>300</v>
+      </c>
+      <c r="C22" s="14">
+        <v>90</v>
+      </c>
+      <c r="D22" s="14">
+        <v>60</v>
+      </c>
+      <c r="E22" s="14">
+        <v>50</v>
+      </c>
+      <c r="F22" s="14">
+        <v>200</v>
+      </c>
+      <c r="G22" s="14">
+        <v>4</v>
+      </c>
+      <c r="H22" s="14">
+        <v>150</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>850</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
+        <v>590</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N22" s="17"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+      <c r="A23" s="8">
+        <v>46262</v>
+      </c>
+      <c r="B23" s="14">
+        <v>420</v>
+      </c>
+      <c r="C23" s="14">
+        <v>100</v>
+      </c>
+      <c r="D23" s="14">
+        <v>60</v>
+      </c>
+      <c r="E23" s="14">
+        <v>50</v>
+      </c>
+      <c r="F23" s="14">
+        <v>250</v>
+      </c>
+      <c r="G23" s="14">
+        <v>5</v>
+      </c>
+      <c r="H23" s="14">
+        <v>130</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
+        <v>430</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="15" t="str">
+      <c r="A24" s="8">
+        <v>46263</v>
+      </c>
+      <c r="B24" s="14">
+        <v>360</v>
+      </c>
+      <c r="C24" s="14">
+        <v>110</v>
+      </c>
+      <c r="D24" s="14">
+        <v>60</v>
+      </c>
+      <c r="E24" s="14">
+        <v>50</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0</v>
+      </c>
+      <c r="H24" s="14">
+        <v>150</v>
+      </c>
+      <c r="I24" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="15" t="str">
+        <v>730</v>
+      </c>
+      <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
+        <v>710</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L24" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N24" s="17"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A25" s="13"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="15" t="str">
+      <c r="A25" s="8">
+        <v>46264</v>
+      </c>
+      <c r="B25" s="14">
+        <v>300</v>
+      </c>
+      <c r="C25" s="14">
+        <v>0</v>
+      </c>
+      <c r="D25" s="14">
+        <v>60</v>
+      </c>
+      <c r="E25" s="14">
+        <v>50</v>
+      </c>
+      <c r="F25" s="14">
+        <v>0</v>
+      </c>
+      <c r="G25" s="14">
+        <v>0</v>
+      </c>
+      <c r="H25" s="14">
+        <v>90</v>
+      </c>
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="15" t="str">
+        <v>500</v>
+      </c>
+      <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
+        <v>940</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N25" s="17"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="13"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="15" t="str">
+      <c r="A26" s="8">
+        <v>46265</v>
+      </c>
+      <c r="B26" s="14">
+        <v>300</v>
+      </c>
+      <c r="C26" s="14">
+        <v>120</v>
+      </c>
+      <c r="D26" s="14">
+        <v>40</v>
+      </c>
+      <c r="E26" s="14">
+        <v>40</v>
+      </c>
+      <c r="F26" s="14">
+        <v>250</v>
+      </c>
+      <c r="G26" s="14">
+        <v>5</v>
+      </c>
+      <c r="H26" s="14">
+        <v>300</v>
+      </c>
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="16"/>
-      <c r="L26" s="16"/>
-      <c r="M26" s="16"/>
+        <v>390</v>
+      </c>
+      <c r="K26" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L26" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N26" s="17"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="15" t="str">
+      <c r="A27" s="8">
+        <v>46266</v>
+      </c>
+      <c r="B27" s="14">
+        <v>300</v>
+      </c>
+      <c r="C27" s="14">
+        <v>120</v>
+      </c>
+      <c r="D27" s="14">
+        <v>45</v>
+      </c>
+      <c r="E27" s="14">
+        <v>40</v>
+      </c>
+      <c r="F27" s="14">
+        <v>350</v>
+      </c>
+      <c r="G27" s="14">
+        <v>7</v>
+      </c>
+      <c r="H27" s="14">
+        <v>100</v>
+      </c>
+      <c r="I27" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="15" t="str">
+        <v>955</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="16"/>
-      <c r="L27" s="16"/>
-      <c r="M27" s="16"/>
+        <v>485</v>
+      </c>
+      <c r="K27" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N27" s="17"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="8">
+        <v>46267</v>
+      </c>
+      <c r="B28" s="14">
+        <v>300</v>
+      </c>
+      <c r="C28" s="14">
+        <v>120</v>
+      </c>
+      <c r="D28" s="14">
+        <v>60</v>
+      </c>
+      <c r="E28" s="14">
+        <v>40</v>
+      </c>
+      <c r="F28" s="14">
+        <v>300</v>
+      </c>
+      <c r="G28" s="14">
+        <v>6</v>
+      </c>
+      <c r="H28" s="14">
+        <v>90</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>910</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
+        <v>530</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N28" s="17"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="15" t="str">
+      <c r="A29" s="8">
+        <v>46268</v>
+      </c>
+      <c r="B29" s="14">
+        <v>300</v>
+      </c>
+      <c r="C29" s="14">
+        <v>90</v>
+      </c>
+      <c r="D29" s="14">
+        <v>0</v>
+      </c>
+      <c r="E29" s="14">
+        <v>100</v>
+      </c>
+      <c r="F29" s="14">
+        <v>200</v>
+      </c>
+      <c r="G29" s="14">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14">
+        <v>200</v>
+      </c>
+      <c r="I29" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="15" t="str">
+        <v>890</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
+        <v>550</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N29" s="17"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="13"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="15" t="str">
+      <c r="A30" s="8">
+        <v>46269</v>
+      </c>
+      <c r="B30" s="14">
+        <v>420</v>
+      </c>
+      <c r="C30" s="14">
+        <v>120</v>
+      </c>
+      <c r="D30" s="14">
+        <v>0</v>
+      </c>
+      <c r="E30" s="14">
+        <v>90</v>
+      </c>
+      <c r="F30" s="14">
+        <v>250</v>
+      </c>
+      <c r="G30" s="14">
+        <v>5</v>
+      </c>
+      <c r="H30" s="14">
+        <v>200</v>
+      </c>
+      <c r="I30" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
+        <v>360</v>
+      </c>
+      <c r="K30" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L30" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M30" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N30" s="17"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="13"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="15" t="str">
+      <c r="A31" s="8">
+        <v>46270</v>
+      </c>
+      <c r="B31" s="14">
+        <v>420</v>
+      </c>
+      <c r="C31" s="14">
+        <v>90</v>
+      </c>
+      <c r="D31" s="14">
+        <v>100</v>
+      </c>
+      <c r="E31" s="14">
+        <v>30</v>
+      </c>
+      <c r="F31" s="14">
+        <v>0</v>
+      </c>
+      <c r="G31" s="14">
+        <v>0</v>
+      </c>
+      <c r="H31" s="14">
+        <v>120</v>
+      </c>
+      <c r="I31" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="15" t="str">
+        <v>760</v>
+      </c>
+      <c r="J31" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
+        <v>680</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N31" s="17"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="13"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="15" t="str">
+      <c r="A32" s="8">
+        <v>46271</v>
+      </c>
+      <c r="B32" s="14">
+        <v>300</v>
+      </c>
+      <c r="C32" s="14">
+        <v>0</v>
+      </c>
+      <c r="D32" s="14">
+        <v>30</v>
+      </c>
+      <c r="E32" s="14">
+        <v>30</v>
+      </c>
+      <c r="F32" s="14">
+        <v>0</v>
+      </c>
+      <c r="G32" s="14">
+        <v>0</v>
+      </c>
+      <c r="H32" s="14">
+        <v>300</v>
+      </c>
+      <c r="I32" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="15" t="str">
+        <v>660</v>
+      </c>
+      <c r="J32" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
+        <v>780</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L32" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M32" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N32" s="17"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+      <c r="A33" s="8">
+        <v>46272</v>
+      </c>
+      <c r="B33" s="14">
+        <v>360</v>
+      </c>
+      <c r="C33" s="14">
+        <v>90</v>
+      </c>
+      <c r="D33" s="14">
+        <v>90</v>
+      </c>
+      <c r="E33" s="14">
+        <v>30</v>
+      </c>
+      <c r="F33" s="14">
+        <v>250</v>
+      </c>
+      <c r="G33" s="14">
+        <v>5</v>
+      </c>
+      <c r="H33" s="14">
+        <v>130</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N33" s="17"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+      <c r="A34" s="8">
+        <v>46273</v>
+      </c>
+      <c r="B34" s="14">
+        <v>360</v>
+      </c>
+      <c r="C34" s="14">
+        <v>100</v>
+      </c>
+      <c r="D34" s="14">
+        <v>100</v>
+      </c>
+      <c r="E34" s="14">
+        <v>30</v>
+      </c>
+      <c r="F34" s="14">
+        <v>350</v>
+      </c>
+      <c r="G34" s="14">
+        <v>7</v>
+      </c>
+      <c r="H34" s="14">
+        <v>100</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N34" s="17"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+      <c r="A35" s="8">
+        <v>46274</v>
+      </c>
+      <c r="B35" s="14">
+        <v>360</v>
+      </c>
+      <c r="C35" s="14">
+        <v>95</v>
+      </c>
+      <c r="D35" s="14">
+        <v>120</v>
+      </c>
+      <c r="E35" s="14">
+        <v>20</v>
+      </c>
+      <c r="F35" s="14">
+        <v>300</v>
+      </c>
+      <c r="G35" s="14">
+        <v>6</v>
+      </c>
+      <c r="H35" s="14">
+        <v>110</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1005</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
+        <v>435</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N35" s="17"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="13"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="15" t="str">
+      <c r="A36" s="8">
+        <v>46275</v>
+      </c>
+      <c r="B36" s="14">
+        <v>360</v>
+      </c>
+      <c r="C36" s="14">
+        <v>100</v>
+      </c>
+      <c r="D36" s="14">
+        <v>0</v>
+      </c>
+      <c r="E36" s="14">
+        <v>100</v>
+      </c>
+      <c r="F36" s="14">
+        <v>200</v>
+      </c>
+      <c r="G36" s="14">
+        <v>4</v>
+      </c>
+      <c r="H36" s="14">
+        <v>90</v>
+      </c>
+      <c r="I36" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J36" s="15" t="str">
+        <v>850</v>
+      </c>
+      <c r="J36" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K36" s="16"/>
-      <c r="L36" s="16"/>
-      <c r="M36" s="16"/>
+        <v>590</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L36" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N36" s="17"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+      <c r="A37" s="8">
+        <v>46276</v>
+      </c>
+      <c r="B37" s="14">
+        <v>420</v>
+      </c>
+      <c r="C37" s="14">
+        <v>110</v>
+      </c>
+      <c r="D37" s="14">
+        <v>110</v>
+      </c>
+      <c r="E37" s="14">
+        <v>90</v>
+      </c>
+      <c r="F37" s="14">
+        <v>250</v>
+      </c>
+      <c r="G37" s="14">
+        <v>5</v>
+      </c>
+      <c r="H37" s="14">
+        <v>90</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>1070</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
+        <v>370</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N37" s="17"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+      <c r="A38" s="8">
+        <v>46277</v>
+      </c>
+      <c r="B38" s="14">
+        <v>420</v>
+      </c>
+      <c r="C38" s="14">
+        <v>90</v>
+      </c>
+      <c r="D38" s="14">
+        <v>90</v>
+      </c>
+      <c r="E38" s="14">
+        <v>20</v>
+      </c>
+      <c r="F38" s="14">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14">
+        <v>300</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
+        <v>520</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N38" s="17"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+      <c r="A39" s="8">
+        <v>46278</v>
+      </c>
+      <c r="B39" s="14">
+        <v>360</v>
+      </c>
+      <c r="C39" s="14">
+        <v>0</v>
+      </c>
+      <c r="D39" s="14">
+        <v>0</v>
+      </c>
+      <c r="E39" s="14">
+        <v>30</v>
+      </c>
+      <c r="F39" s="14">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14">
+        <v>0</v>
+      </c>
+      <c r="H39" s="14">
+        <v>300</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>690</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
+        <v>750</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N39" s="17"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+      <c r="A40" s="8">
+        <v>46279</v>
+      </c>
+      <c r="B40" s="14">
+        <v>360</v>
+      </c>
+      <c r="C40" s="14">
+        <v>90</v>
+      </c>
+      <c r="D40" s="14">
+        <v>90</v>
+      </c>
+      <c r="E40" s="14">
+        <v>45</v>
+      </c>
+      <c r="F40" s="14">
+        <v>200</v>
+      </c>
+      <c r="G40" s="14">
+        <v>4</v>
+      </c>
+      <c r="H40" s="14">
+        <v>120</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>905</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
+        <v>535</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N40" s="17"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+      <c r="A41" s="8">
+        <v>46280</v>
+      </c>
+      <c r="B41" s="14">
+        <v>360</v>
+      </c>
+      <c r="C41" s="14">
+        <v>110</v>
+      </c>
+      <c r="D41" s="14">
+        <v>90</v>
+      </c>
+      <c r="E41" s="14">
+        <v>0</v>
+      </c>
+      <c r="F41" s="14">
+        <v>300</v>
+      </c>
+      <c r="G41" s="14">
+        <v>6</v>
+      </c>
+      <c r="H41" s="14">
+        <v>120</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>980</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
+        <v>460</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N41" s="17"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="15" t="str">
+      <c r="A42" s="8">
+        <v>46281</v>
+      </c>
+      <c r="B42" s="14">
+        <v>360</v>
+      </c>
+      <c r="C42" s="14">
+        <v>100</v>
+      </c>
+      <c r="D42" s="14">
+        <v>90</v>
+      </c>
+      <c r="E42" s="14">
+        <v>0</v>
+      </c>
+      <c r="F42" s="14">
+        <v>250</v>
+      </c>
+      <c r="G42" s="14">
+        <v>5</v>
+      </c>
+      <c r="H42" s="14">
+        <v>150</v>
+      </c>
+      <c r="I42" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J42" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J42" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K42" s="16"/>
-      <c r="L42" s="16"/>
-      <c r="M42" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K42" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N42" s="17"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A43" s="13"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="15" t="str">
+      <c r="A43" s="8">
+        <v>46282</v>
+      </c>
+      <c r="B43" s="14">
+        <v>360</v>
+      </c>
+      <c r="C43" s="14">
+        <v>90</v>
+      </c>
+      <c r="D43" s="14">
+        <v>90</v>
+      </c>
+      <c r="E43" s="14">
+        <v>30</v>
+      </c>
+      <c r="F43" s="14">
+        <v>150</v>
+      </c>
+      <c r="G43" s="14">
+        <v>3</v>
+      </c>
+      <c r="H43" s="14">
+        <v>180</v>
+      </c>
+      <c r="I43" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J43" s="15" t="str">
+        <v>900</v>
+      </c>
+      <c r="J43" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="16"/>
-      <c r="M43" s="16"/>
+        <v>540</v>
+      </c>
+      <c r="K43" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L43" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M43" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N43" s="17"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A44" s="13"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="15" t="str">
+      <c r="A44" s="8">
+        <v>46283</v>
+      </c>
+      <c r="B44" s="14">
+        <v>420</v>
+      </c>
+      <c r="C44" s="14">
+        <v>45</v>
+      </c>
+      <c r="D44" s="14">
+        <v>45</v>
+      </c>
+      <c r="E44" s="14">
+        <v>40</v>
+      </c>
+      <c r="F44" s="14">
+        <v>250</v>
+      </c>
+      <c r="G44" s="14">
+        <v>5</v>
+      </c>
+      <c r="H44" s="14">
+        <v>300</v>
+      </c>
+      <c r="I44" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J44" s="15" t="str">
+        <v>1100</v>
+      </c>
+      <c r="J44" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K44" s="16"/>
-      <c r="L44" s="16"/>
-      <c r="M44" s="16"/>
+        <v>340</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L44" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M44" s="16" t="s">
+        <v>58</v>
+      </c>
       <c r="N44" s="17"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14"/>
-      <c r="C45" s="14"/>
-      <c r="D45" s="14"/>
-      <c r="E45" s="14"/>
-      <c r="F45" s="14"/>
-      <c r="G45" s="14"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="15" t="str">
+      <c r="A45" s="8">
+        <v>46284</v>
+      </c>
+      <c r="B45" s="14">
+        <v>420</v>
+      </c>
+      <c r="C45" s="14">
+        <v>60</v>
+      </c>
+      <c r="D45" s="14">
+        <v>90</v>
+      </c>
+      <c r="E45" s="14">
+        <v>0</v>
+      </c>
+      <c r="F45" s="14">
+        <v>0</v>
+      </c>
+      <c r="G45" s="14">
+        <v>0</v>
+      </c>
+      <c r="H45" s="14">
+        <v>300</v>
+      </c>
+      <c r="I45" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J45" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J45" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="16"/>
-      <c r="M45" s="16"/>
+        <v>570</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L45" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M45" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N45" s="17"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A46" s="13"/>
-      <c r="B46" s="14"/>
-      <c r="C46" s="14"/>
-      <c r="D46" s="14"/>
-      <c r="E46" s="14"/>
-      <c r="F46" s="14"/>
-      <c r="G46" s="14"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="15" t="str">
+      <c r="A46" s="8">
+        <v>46285</v>
+      </c>
+      <c r="B46" s="14">
+        <v>360</v>
+      </c>
+      <c r="C46" s="14">
+        <v>0</v>
+      </c>
+      <c r="D46" s="14">
+        <v>90</v>
+      </c>
+      <c r="E46" s="14">
+        <v>90</v>
+      </c>
+      <c r="F46" s="14">
+        <v>0</v>
+      </c>
+      <c r="G46" s="14">
+        <v>0</v>
+      </c>
+      <c r="H46" s="14">
+        <v>300</v>
+      </c>
+      <c r="I46" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J46" s="15" t="str">
+        <v>840</v>
+      </c>
+      <c r="J46" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K46" s="16"/>
-      <c r="L46" s="16"/>
-      <c r="M46" s="16"/>
+        <v>600</v>
+      </c>
+      <c r="K46" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L46" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="M46" s="16" t="s">
+        <v>49</v>
+      </c>
       <c r="N46" s="17"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>